<commit_message>
it works for the first page so far
</commit_message>
<xml_diff>
--- a/cars_and_bids.xlsx
+++ b/cars_and_bids.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X16"/>
+  <dimension ref="A1:X26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,45 +541,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/rN5QjdWK/2020-aston-martin-db11-coupe</t>
+          <t>https://carsandbids.com/auctions/K1xDejkd/2008-porsche-911-turbo-coupe</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2020 Aston Martin DB11 Coupe VIN: SCFRMFAW8LGL09276 for Sale - Cars &amp; Bids</t>
+          <t>2008 Porsche 911 Turbo Coupe VIN: WP0AD29918S783562 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Aston Martin</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DB11Save</t>
+          <t>997 911Save</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.0L Turbocharged V8</t>
+          <t>3.6L Turbocharged Flat-6</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rear-wheel drive</t>
+          <t>4WD/AWD</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>34900</v>
+        <v>76300</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Automatic (8-Speed)</t>
+          <t>Manual (6-Speed)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SCFRMFAW8LGL09276</t>
+          <t>WP0AD29918S783562</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -589,37 +589,37 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Rebuilt (IN)</t>
+          <t>Clean (SC)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Meteor Grey Metallic</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Black/Stone Grey</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Glenview</t>
+          <t>Folly Beach</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>60025</t>
+          <t>29439</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Dpiecha21</t>
+          <t>JDOFOSHO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -629,107 +629,109 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Bid to$51,500</t>
+          <t>Sold for$93,000</t>
         </is>
       </c>
       <c r="T2" t="n">
-        <v>51500</v>
+        <v>93000</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:54 PM MDT</t>
+          <t>Apr 30, 2026 2:08 PM MDT</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="W2" t="n">
-        <v>7914</v>
+        <v>12628</v>
       </c>
       <c r="X2" t="n">
-        <v>706</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/rxRjgyG0/1989-nissan-240sx</t>
+          <t>https://carsandbids.com/auctions/9W1MPw75/2002-toyota-4runner-sr5-4x4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1989 Nissan 240SX VIN: JN1HS36P8KW003377 for Sale - Cars &amp; Bids</t>
+          <t>2002 Toyota 4Runner SR5 4x4 VIN: JT3HN86R320386445 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>240SXSave</t>
+          <t>4RunnerSave</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2.0L Turbocharged I4</t>
+          <t>3.4L V6</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rear-wheel drive</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>4WD/AWD</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>165400</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Manual (5-Speed)</t>
+          <t>Automatic (4-Speed)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>JN1HS36P8KW003377</t>
+          <t>JT3HN86R320386445</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Coupe</t>
+          <t>SUV/Crossover</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Clean (TN)</t>
+          <t>Clean (VA)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Blue-Green Pearl</t>
+          <t>Millennium Silver</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Oak</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Chattanooga</t>
+          <t>Bethesda</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>37415</t>
+          <t>20817</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>micmac2869</t>
+          <t>Aircooledjames</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -739,84 +741,84 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Sold for$11,600</t>
+          <t>Sold for$10,500</t>
         </is>
       </c>
       <c r="T3" t="n">
-        <v>11600</v>
+        <v>10500</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:53 PM MDT</t>
+          <t>Apr 30, 2026 2:03 PM MDT</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="W3" t="n">
-        <v>8467</v>
+        <v>7885</v>
       </c>
       <c r="X3" t="n">
-        <v>520</v>
+        <v>543</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/rbo1npWd/2017-ford-f-150-raptor</t>
+          <t>https://carsandbids.com/auctions/rN5QjdWK/2020-aston-martin-db11-coupe</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2017 Ford F-150 Raptor VIN: 1FTFW1RG9HFB65844 for Sale - Cars &amp; Bids</t>
+          <t>2020 Aston Martin DB11 Coupe VIN: SCFRMFAW8LGL09276 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ford</t>
+          <t>Aston Martin</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>F-150 RaptorSave</t>
+          <t>DB11Save</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3.5L Turbocharged V6</t>
+          <t>4.0L Turbocharged V8</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4WD/AWD</t>
+          <t>Rear-wheel drive</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>75300</v>
+        <v>34900</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Automatic (10-Speed)</t>
+          <t>Automatic (8-Speed)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1FTFW1RG9HFB65844</t>
+          <t>SCFRMFAW8LGL09276</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Truck</t>
+          <t>Coupe</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Clean (TX)</t>
+          <t>Rebuilt (IN)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Magnetic</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -826,22 +828,22 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Glenview</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>78240</t>
+          <t>60025</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>RobertBeka</t>
+          <t>Dpiecha21</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -851,163 +853,161 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Sold for$36,000</t>
+          <t>Bid to$51,500</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>36000</v>
+        <v>51500</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:47 PM MDT</t>
+          <t>Apr 30, 2026 1:54 PM MDT</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="W4" t="n">
-        <v>4202</v>
+        <v>7914</v>
       </c>
       <c r="X4" t="n">
-        <v>381</v>
+        <v>706</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/rjY5z247/2021-subaru-wrx-sti</t>
+          <t>https://carsandbids.com/auctions/rxRjgyG0/1989-nissan-240sx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2021 Subaru WRX STI VIN: JF1VA2E66M9820246 for Sale - Cars &amp; Bids</t>
+          <t>1989 Nissan 240SX VIN: JN1HS36P8KW003377 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Subaru</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>WRX STISave</t>
+          <t>240SXSave</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2.5L Turbocharged Flat-4</t>
+          <t>2.0L Turbocharged I4</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4WD/AWD</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>9700</v>
-      </c>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Manual (6-Speed)</t>
+          <t>Manual (5-Speed)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>JF1VA2E66M9820246</t>
+          <t>JN1HS36P8KW003377</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sedan</t>
+          <t>Coupe</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Clean (CO)</t>
+          <t>Clean (TN)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Magnetite Gray Metallic</t>
+          <t>Blue-Green Pearl</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Black/Red</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Chattanooga</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>80237</t>
+          <t>37415</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>aymen_el</t>
+          <t>micmac2869</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>No Reserve</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Bid to$34,100</t>
+          <t>Sold for$11,600</t>
         </is>
       </c>
       <c r="T5" t="n">
-        <v>34100</v>
+        <v>11600</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:42 PM MDT</t>
+          <t>Apr 30, 2026 1:53 PM MDT</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="W5" t="n">
-        <v>4508</v>
+        <v>8467</v>
       </c>
       <c r="X5" t="n">
-        <v>356</v>
+        <v>517</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/92DpRexK/2014-mercedes-benz-cls550-4matic</t>
+          <t>https://carsandbids.com/auctions/rbo1npWd/2017-ford-f-150-raptor</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2014 Mercedes-Benz CLS550 4Matic VIN: WDDLJ9BB6EA116730 for Sale - Cars &amp; Bids</t>
+          <t>2017 Ford F-150 Raptor VIN: 1FTFW1RG9HFB65844 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Ford</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CLS-ClassSave</t>
+          <t>F-150 RaptorSave</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4.7L Turbocharged V8</t>
+          <t>3.5L Turbocharged V6</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1016,110 +1016,110 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>116900</v>
+        <v>75300</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Automatic (7-Speed)</t>
+          <t>Automatic (10-Speed)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>WDDLJ9BB6EA116730</t>
+          <t>1FTFW1RG9HFB65844</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sedan</t>
+          <t>Truck</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Clean (OH)</t>
+          <t>Clean (TX)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>Magnetic</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Black</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Harrison</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>45030</t>
+          <t>78240</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>rogurts</t>
+          <t>RobertBeka</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>No Reserve</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Sold for$11,259</t>
+          <t>Sold for$36,000</t>
         </is>
       </c>
       <c r="T6" t="n">
-        <v>11259</v>
+        <v>36000</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:40 PM MDT</t>
+          <t>Apr 30, 2026 1:47 PM MDT</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="W6" t="n">
-        <v>5671</v>
+        <v>4202</v>
       </c>
       <c r="X6" t="n">
-        <v>412</v>
+        <v>380</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/9eaZl8yd/2021-jeep-gladiator-rubicon-4x4</t>
+          <t>https://carsandbids.com/auctions/rjY5z247/2021-subaru-wrx-sti</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2021 Jeep Gladiator Rubicon 4x4 VIN: 1C6JJTBM5ML503568 for Sale - Cars &amp; Bids</t>
+          <t>2021 Subaru WRX STI VIN: JF1VA2E66M9820246 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jeep</t>
+          <t>Subaru</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GladiatorSave</t>
+          <t>WRX STISave</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.0L Turbodiesel V6</t>
+          <t>2.5L Turbocharged Flat-4</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1128,56 +1128,56 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>87000</v>
+        <v>9700</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Automatic (8-Speed)</t>
+          <t>Manual (6-Speed)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1C6JJTBM5ML503568</t>
+          <t>JF1VA2E66M9820246</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Truck</t>
+          <t>Sedan</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Clean (NH)</t>
+          <t>Clean (CO)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Granite Crystal Metallic</t>
+          <t>Magnetite Gray Metallic</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Black/Red</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Framingham</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>01701</t>
+          <t>80237</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>KoIneosGrenadier</t>
+          <t>aymen_el</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1187,60 +1187,60 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Bid to$23,000</t>
+          <t>Bid to$34,100</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>23000</v>
+        <v>34100</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:34 PM MDT</t>
+          <t>Apr 30, 2026 1:42 PM MDT</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W7" t="n">
-        <v>2999</v>
+        <v>4508</v>
       </c>
       <c r="X7" t="n">
-        <v>243</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/9lakqNJm/2023-volkswagen-gti-40th-anniversary-edition</t>
+          <t>https://carsandbids.com/auctions/92DpRexK/2014-mercedes-benz-cls550-4matic</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2023 Volkswagen GTI 40th Anniversary Edition VIN: WVW4A7CD4PW159195 for Sale - Cars &amp; Bids</t>
+          <t>2014 Mercedes-Benz CLS550 4Matic VIN: WDDLJ9BB6EA116730 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Volkswagen</t>
+          <t>Mercedes-Benz</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mk8 GTISave</t>
+          <t>CLS-ClassSave</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2.0L Turbocharged I4</t>
+          <t>4.7L Turbocharged V8</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Front-wheel drive</t>
+          <t>4WD/AWD</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>13400</v>
+        <v>116900</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1249,134 +1249,134 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>WVW4A7CD4PW159195</t>
+          <t>WDDLJ9BB6EA116730</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Hatchback</t>
+          <t>Sedan</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Clean (CA)</t>
+          <t>Clean (OH)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Urano Gray</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Titan Black/Plaid</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Fremont</t>
+          <t>Harrison</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>94538</t>
+          <t>45030</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Devin6788</t>
+          <t>rogurts</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>No Reserve</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Bid to$25,750</t>
+          <t>Sold for$11,259</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>25750</v>
+        <v>11259</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:33 PM MDT</t>
+          <t>Apr 30, 2026 1:40 PM MDT</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="W8" t="n">
-        <v>4904</v>
+        <v>5671</v>
       </c>
       <c r="X8" t="n">
-        <v>371</v>
+        <v>412</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/K1Aap6d2/2011-porsche-cayman-s</t>
+          <t>https://carsandbids.com/auctions/9eaZl8yd/2021-jeep-gladiator-rubicon-4x4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2011 Porsche Cayman S VIN: WP0AB2A8XBU780535 for Sale - Cars &amp; Bids</t>
+          <t>2021 Jeep Gladiator Rubicon 4x4 VIN: 1C6JJTBM5ML503568 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Jeep</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>987 CaymanSave</t>
+          <t>GladiatorSave</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3.4L Flat-6</t>
+          <t>3.0L Turbodiesel V6</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rear-wheel drive</t>
+          <t>4WD/AWD</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>31700</v>
+        <v>87000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Manual (6-Speed)</t>
+          <t>Automatic (8-Speed)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>WP0AB2A8XBU780535</t>
+          <t>1C6JJTBM5ML503568</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Coupe</t>
+          <t>Truck</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Clean (TN)</t>
+          <t>Clean (NH)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Meteor Grey Metallic</t>
+          <t>Granite Crystal Metallic</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1386,22 +1386,22 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Church Hill</t>
+          <t>Framingham</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>37642</t>
+          <t>01701</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>KUHL_9872</t>
+          <t>KoIneosGrenadier</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1411,51 +1411,51 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Sold for$59,500</t>
+          <t>Bid to$23,000</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>59500</v>
+        <v>23000</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:31 PM MDT</t>
+          <t>Apr 30, 2026 1:34 PM MDT</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="W9" t="n">
-        <v>9750</v>
+        <v>2999</v>
       </c>
       <c r="X9" t="n">
-        <v>928</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/37QOoW47/2015-mini-cooper-hardtop</t>
+          <t>https://carsandbids.com/auctions/9lakqNJm/2023-volkswagen-gti-40th-anniversary-edition</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2015 Mini Cooper Hardtop VIN: WMWXM5C51F3A97577 for Sale - Cars &amp; Bids</t>
+          <t>2023 Volkswagen GTI 40th Anniversary Edition VIN: WVW4A7CD4PW159195 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MINI</t>
+          <t>Volkswagen</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CooperSave</t>
+          <t>Mk8 GTISave</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5L Turbocharged I3</t>
+          <t>2.0L Turbocharged I4</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1464,16 +1464,16 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>149000</v>
+        <v>13400</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Manual (6-Speed)</t>
+          <t>Automatic (7-Speed)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>WMWXM5C51F3A97577</t>
+          <t>WVW4A7CD4PW159195</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1483,539 +1483,539 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Clean (CT)</t>
+          <t>Clean (CA)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Volcanic Orange</t>
+          <t>Urano Gray</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Carbon Black</t>
+          <t>Titan Black/Plaid</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Wallingford</t>
+          <t>Fremont</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>06492</t>
+          <t>94538</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>PSQ</t>
+          <t>Devin6788</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>No Reserve</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Sold for$5,500</t>
+          <t>Bid to$25,750</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>5500</v>
+        <v>25750</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:29 PM MDT</t>
+          <t>Apr 30, 2026 1:33 PM MDT</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W10" t="n">
-        <v>4369</v>
+        <v>4904</v>
       </c>
       <c r="X10" t="n">
-        <v>312</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/KZJ41Bjm/2016-volkswagen-golf-sportwagen-se</t>
+          <t>https://carsandbids.com/auctions/K1Aap6d2/2011-porsche-cayman-s</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2016 Volkswagen Golf SportWagen SE VIN: 3VWC17AU1GM507935 for Sale - Cars &amp; Bids</t>
+          <t>2011 Porsche Cayman S VIN: WP0AB2A8XBU780535 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Volkswagen</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GolfSave</t>
+          <t>987 CaymanSave</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.8L Turbocharged I4</t>
+          <t>3.4L Flat-6</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Front-wheel drive</t>
+          <t>Rear-wheel drive</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>81500</v>
+        <v>31700</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Automatic (6-Speed)</t>
+          <t>Manual (6-Speed)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3VWC17AU1GM507935</t>
+          <t>WP0AB2A8XBU780535</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Wagon</t>
+          <t>Coupe</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Clean (GA)</t>
+          <t>Clean (TN)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Platinum Gray Metallic</t>
+          <t>Meteor Grey Metallic</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Titan Black</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Buford</t>
+          <t>Church Hill</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>30519</t>
+          <t>37642</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>GaDeluxeMotors</t>
+          <t>KUHL_9872</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>No Reserve</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Sold for$10,100</t>
+          <t>Sold for$59,500</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>10100</v>
+        <v>59500</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:20 PM MDT</t>
+          <t>Apr 30, 2026 1:31 PM MDT</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="W11" t="n">
-        <v>4590</v>
+        <v>9750</v>
       </c>
       <c r="X11" t="n">
-        <v>355</v>
+        <v>927</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/rjqLX6Rl/2018-audi-q7-premium-plus</t>
+          <t>https://carsandbids.com/auctions/37QOoW47/2015-mini-cooper-hardtop</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2018 Audi Q7 Premium Plus VIN: WA1LAAF78JD003530 for Sale - Cars &amp; Bids</t>
+          <t>2015 Mini Cooper Hardtop VIN: WMWXM5C51F3A97577 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>MINI</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Q7Save</t>
+          <t>CooperSave</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3.0L Supercharged V6</t>
+          <t>1.5L Turbocharged I3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>4WD/AWD</t>
+          <t>Front-wheel drive</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>79200</v>
+        <v>149000</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Automatic (8-Speed)</t>
+          <t>Manual (6-Speed)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>WA1LAAF78JD003530</t>
+          <t>WMWXM5C51F3A97577</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>SUV/Crossover</t>
+          <t>Hatchback</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Clean (TX)</t>
+          <t>Clean (CT)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Glacier White Metallic</t>
+          <t>Volcanic Orange</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Pistachio Beige</t>
+          <t>Carbon Black</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Wallingford</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>77042</t>
+          <t>06492</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>UnitedExpressAuto</t>
+          <t>PSQ</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>No Reserve</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Sold for$18,500</t>
+          <t>Sold for$5,500</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>18500</v>
+        <v>5500</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:17 PM MDT</t>
+          <t>Apr 30, 2026 1:29 PM MDT</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="W12" t="n">
-        <v>3804</v>
+        <v>4369</v>
       </c>
       <c r="X12" t="n">
-        <v>298</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/3y2YePZp/2015-chevrolet-corvette-stingray-coupe</t>
+          <t>https://carsandbids.com/auctions/KZJ41Bjm/2016-volkswagen-golf-sportwagen-se</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2015 Chevrolet Corvette Stingray Coupe VIN: 1G1YE2D76F5105377 for Sale - Cars &amp; Bids</t>
+          <t>2016 Volkswagen Golf SportWagen SE VIN: 3VWC17AU1GM507935 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chevrolet</t>
+          <t>Volkswagen</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C7 CorvetteSave</t>
+          <t>GolfSave</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6.2L V8</t>
+          <t>1.8L Turbocharged I4</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rear-wheel drive</t>
+          <t>Front-wheel drive</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>38900</v>
+        <v>81500</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Manual (7-Speed)</t>
+          <t>Automatic (6-Speed)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1G1YE2D76F5105377</t>
+          <t>3VWC17AU1GM507935</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Coupe</t>
+          <t>Wagon</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Clean (TX)</t>
+          <t>Clean (GA)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Laguna Blue Tintcoat</t>
+          <t>Platinum Gray Metallic</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Gray</t>
+          <t>Titan Black</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Palo Pinto</t>
+          <t>Buford</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>76484</t>
+          <t>30519</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>DW1811</t>
+          <t>GaDeluxeMotors</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>No Reserve</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Sold for$40,000</t>
+          <t>Sold for$10,100</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>40000</v>
+        <v>10100</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:17 PM MDT</t>
+          <t>Apr 30, 2026 1:20 PM MDT</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="W13" t="n">
-        <v>5834</v>
+        <v>4590</v>
       </c>
       <c r="X13" t="n">
-        <v>664</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/9WoM1wgB/2000-porsche-boxster-s</t>
+          <t>https://carsandbids.com/auctions/rjqLX6Rl/2018-audi-q7-premium-plus</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2000 Porsche Boxster S VIN: WP0CB2985YU662978 for Sale - Cars &amp; Bids</t>
+          <t>2018 Audi Q7 Premium Plus VIN: WA1LAAF78JD003530 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>986 BoxsterSave</t>
+          <t>Q7Save</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3.2L Flat-6</t>
+          <t>3.0L Supercharged V6</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Rear-wheel drive</t>
+          <t>4WD/AWD</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>96800</v>
+        <v>79200</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Manual (6-Speed)</t>
+          <t>Automatic (8-Speed)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>WP0CB2985YU662978</t>
+          <t>WA1LAAF78JD003530</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Convertible</t>
+          <t>SUV/Crossover</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Clean (CA)</t>
+          <t>Clean (TX)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Glacier White Metallic</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Pistachio Beige</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Lathrop</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>95330</t>
+          <t>77042</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>longimotorsports</t>
+          <t>UnitedExpressAuto</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>No Reserve</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Sold for$12,300</t>
+          <t>Sold for$18,500</t>
         </is>
       </c>
       <c r="T14" t="n">
-        <v>12300</v>
+        <v>18500</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:06 PM MDT</t>
+          <t>Apr 30, 2026 1:17 PM MDT</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="W14" t="n">
-        <v>5770</v>
+        <v>3804</v>
       </c>
       <c r="X14" t="n">
-        <v>539</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://carsandbids.com/auctions/3vEJmGRj/2008-bmw-m3-coupe</t>
+          <t>https://carsandbids.com/auctions/3y2YePZp/2015-chevrolet-corvette-stingray-coupe</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2008 BMW M3 Coupe VIN: WBSWD93518PY41931 for Sale - Cars &amp; Bids</t>
+          <t>2015 Chevrolet Corvette Stingray Coupe VIN: 1G1YE2D76F5105377 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Chevrolet</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>E9X M3Save</t>
+          <t>C7 CorvetteSave</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4.0L V8</t>
+          <t>6.2L V8</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2024,16 +2024,16 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>89400</v>
+        <v>38900</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Manual (6-Speed)</t>
+          <t>Manual (7-Speed)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>WBSWD93518PY41931</t>
+          <t>1G1YE2D76F5105377</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2043,37 +2043,37 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Clean (TN)</t>
+          <t>Clean (TX)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Sparkling Graphite Metallic</t>
+          <t>Laguna Blue Tintcoat</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Gray</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Eads</t>
+          <t>Palo Pinto</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>38028</t>
+          <t>76484</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>rokas</t>
+          <t>DW1811</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2083,137 +2083,1255 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Bid to$27,000</t>
+          <t>Sold for$40,000</t>
         </is>
       </c>
       <c r="T15" t="n">
-        <v>27000</v>
+        <v>40000</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:02 PM MDT</t>
+          <t>Apr 30, 2026 1:17 PM MDT</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="W15" t="n">
-        <v>7433</v>
+        <v>5834</v>
       </c>
       <c r="X15" t="n">
-        <v>605</v>
+        <v>663</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>https://carsandbids.com/auctions/9WoM1wgB/2000-porsche-boxster-s</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2000 Porsche Boxster S VIN: WP0CB2985YU662978 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Porsche</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>986 BoxsterSave</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>3.2L Flat-6</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>96800</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Manual (6-Speed)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>WP0CB2985YU662978</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Clean (CA)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Lathrop</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>95330</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>longimotorsports</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>No Reserve</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Sold for$12,300</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>12300</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 1:06 PM MDT</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>15</v>
+      </c>
+      <c r="W16" t="n">
+        <v>5770</v>
+      </c>
+      <c r="X16" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/3vEJmGRj/2008-bmw-m3-coupe</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2008 BMW M3 Coupe VIN: WBSWD93518PY41931 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BMW</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>E9X M3Save</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4.0L V8</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>89400</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Manual (6-Speed)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>WBSWD93518PY41931</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Coupe</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Clean (TN)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Sparkling Graphite Metallic</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Eads</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>38028</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>rokas</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Bid to$27,000</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>27000</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 1:02 PM MDT</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>15</v>
+      </c>
+      <c r="W17" t="n">
+        <v>7433</v>
+      </c>
+      <c r="X17" t="n">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>https://carsandbids.com/auctions/KPmmmBWk/2025-chevrolet-silverado-1500-crew-cab-rst-sherrod-eclipse-4x4</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>2025 Chevrolet Silverado 1500 Crew Cab RST Sherrod Eclipse 4x4 VIN: 3GCUKEE88SG291613 for Sale - Cars &amp; Bids</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Chevrolet</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>SilveradoSave</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>3.0L Turbodiesel I6</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>4WD/AWD</t>
         </is>
       </c>
-      <c r="G16" t="n">
+      <c r="G18" t="n">
         <v>12200</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Automatic (10-Speed)</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>3GCUKEE88SG291613</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Truck</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Clean (FL)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Slate Gray Metallic</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Jet Black</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Miami</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>33177</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>moisesD_F80</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>Bid to$49,000</t>
         </is>
       </c>
-      <c r="T16" t="n">
+      <c r="T18" t="n">
         <v>49000</v>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Apr 30, 2026 1:02 PM MDT</t>
         </is>
       </c>
-      <c r="V16" t="n">
+      <c r="V18" t="n">
         <v>31</v>
       </c>
-      <c r="W16" t="n">
+      <c r="W18" t="n">
         <v>3193</v>
       </c>
-      <c r="X16" t="n">
-        <v>182</v>
+      <c r="X18" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/366Pq8P3/2004-bmw-325xi-touring</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2004 BMW 325xi Touring VIN: WBAEP33424PF04709 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BMW</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3 SeriesSave</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2.5L I6</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>4WD/AWD</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>150400</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Manual (6-Speed)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>WBAEP33424PF04709</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Wagon</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Clean (IL)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Silver Grey Metallic</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>60642</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>patarkimbap</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>No Reserve</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Sold for$3,800</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>3800</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:55 PM MDT</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>13</v>
+      </c>
+      <c r="W19" t="n">
+        <v>7188</v>
+      </c>
+      <c r="X19" t="n">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/rJBxbw7z/2009-mercedes-benz-c63-amg-sedan</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2009 Mercedes-Benz C63 AMG Sedan VIN: WDDGF77X19F330299 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>C-Class AMGSave</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>6.2L V8</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>129000</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Automatic (7-Speed)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>WDDGF77X19F330299</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Sedan</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Clean (GA)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>30328</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>krisrepka</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Bid to$8,250</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>8250</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:52 PM MDT</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>10</v>
+      </c>
+      <c r="W20" t="n">
+        <v>4838</v>
+      </c>
+      <c r="X20" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/KPZqePD7/2021-ford-bronco-black-diamond-advanced</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2021 Ford Bronco Black Diamond Advanced VIN: 1FMEE5DP0MLA74191 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BroncoSave</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2.7L Turbocharged V6</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>4WD/AWD</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>45200</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Automatic (10-Speed)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1FMEE5DP0MLA74191</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SUV/Crossover</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Clean (NJ)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Velocity Blue Metallic</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Gray/Black</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Salt Lake City</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>84106</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>depluber</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Bid to$27,500</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>27500</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:48 PM MDT</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>52</v>
+      </c>
+      <c r="W21" t="n">
+        <v>4113</v>
+      </c>
+      <c r="X21" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/3zW75qMJ/2014-land-rover-lr4-hse-lux</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2014 Land Rover LR4 HSE LUX VIN: SALAK2V6XEA722321 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Land Rover</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LR4Save</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>3.0L Supercharged V6</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>4WD/AWD</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>124000</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Automatic (8-Speed)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SALAK2V6XEA722321</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SUV/Crossover</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Clean (PA)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Santorini Black</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Ebony/Cirrus Grey</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>King Of Prussia</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>19406</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>MotorcarsOfTheMainLine</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Sold for$15,000</t>
+        </is>
+      </c>
+      <c r="T22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:45 PM MDT</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>47</v>
+      </c>
+      <c r="W22" t="n">
+        <v>4484</v>
+      </c>
+      <c r="X22" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/rGYn1D74/2010-mercedes-benz-e550-sedan</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2010 Mercedes-Benz E550 Sedan VIN: WDDHF7CB6AA190895 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>E-ClassSave</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>5.5L V8</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>99200</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Automatic (7-Speed)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>WDDHF7CB6AA190895</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Sedan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Clean (CA)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Calcite White</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Beige</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>90007</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Autoconnections</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>No Reserve</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Sold for$8,500</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
+        <v>8500</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:44 PM MDT</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>19</v>
+      </c>
+      <c r="W23" t="n">
+        <v>4490</v>
+      </c>
+      <c r="X23" t="n">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/3gG40d2y/1992-lexus-es-300</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1992 Lexus ES 300 VIN: JT8VK13T2N0027458 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Lexus</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ESSave</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3.0L V6</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Front-wheel drive</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Manual (5-Speed)</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>JT8VK13T2N0027458</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Sedan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Clean (MN)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Black Onyx</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Isanti</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>55040</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Ian</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>No Reserve</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Sold for$6,300</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>6300</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:35 PM MDT</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>36</v>
+      </c>
+      <c r="W24" t="n">
+        <v>10301</v>
+      </c>
+      <c r="X24" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/3OWl00qm/2024-chevrolet-corvette-stingray-convertible-2lt</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2024 Chevrolet Corvette Stingray Convertible 2LT VIN: 1G1YB3D43R5118967 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>C8 CorvetteSave</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>6.2L V8</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Rear-wheel drive</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>11200</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Automatic (8-Speed)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1G1YB3D43R5118967</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Clean (CA)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Sea Wolf Gray Tricoat</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Adrenaline Red</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Hacienda Heights</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>91745</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Seanyoung</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Bid to$68,000</t>
+        </is>
+      </c>
+      <c r="T25" t="n">
+        <v>68000</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:34 PM MDT</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>33</v>
+      </c>
+      <c r="W25" t="n">
+        <v>6338</v>
+      </c>
+      <c r="X25" t="n">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>https://carsandbids.com/auctions/r40A0XlV/2023-mercedes-amg-e53-cabriolet</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2023 Mercedes-AMG E53 Cabriolet VIN: W1K1K6BB3PF192141 for Sale - Cars &amp; Bids</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>E-Class AMGSave</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3.0L Turbocharged I6</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>4WD/AWD</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>26900</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Automatic (9-Speed)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>W1K1K6BB3PF192141</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Convertible</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Clean (FL)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Obsidian Black Metallic</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Gray</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>33132</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>nistar</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Bid to$55,000</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>55000</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Apr 30, 2026 12:30 PM MDT</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>48</v>
+      </c>
+      <c r="W26" t="n">
+        <v>5577</v>
+      </c>
+      <c r="X26" t="n">
+        <v>454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>